<commit_message>
Rewrite Export Check for human use
Rename and rewrite the first new resource around the plain question a person actually has, remove internal testing language from the public experience, simplify workbook labels and preserve the existing safety limits and resource-specific licence.
</commit_message>
<xml_diff>
--- a/templates/export-recovery-rehearsal/rehearsal.xlsx
+++ b/templates/export-recovery-rehearsal/rehearsal.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Example'!$A$1:$H$25</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Sources and Limits'!$A$1:$H$26</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -198,6 +198,9 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -724,13 +727,6 @@
           <t>Eterna Clarity</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -745,21 +741,14 @@
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Export and Recovery Rehearsal</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
+          <t>Export Check: Can I Still Use My Data?</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Can you do the next useful thing with what you exported?</t>
+          <t>Before you cancel an app, trust a backup, or move your information, check whether the things you actually need still work.</t>
         </is>
       </c>
     </row>
@@ -776,16 +765,9 @@
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Use one workbook for one export or migration. Keep the originals. This worksheet records your observations; it does not export, restore, inspect files, verify permissions or authorise deletion.</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
+          <t>Use one workbook for one export or move. Keep the originals. This checklist does not inspect your files automatically or tell you when it is safe to delete an account.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -800,42 +782,35 @@
     <row r="8" ht="29" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Start with one real task</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
+          <t>Start with one thing you really need to do</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="37" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>1. Choose a task you would need to complete if the source app were unavailable. Identify the records, attachments, links, reminders and access it requires.</t>
+          <t>1. Pick one real task you would need to do if the old app was unavailable, such as finding a document and its attachment or handing a task to someone else.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="37" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2. Make an authorised export. Record the scope and destination on Checks. Do not change or delete original records to test a recovery.</t>
+          <t>2. Export the information you need and keep the original copy. Write down what you exported and where you are moving or storing it.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="43" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>3. Open or import representative material in a separate, permitted test location. Check one example from each relevant area. Use the intended receiver's actual access, not your own logged-in session.</t>
+          <t>3. Open a few real examples. Check the files, attachments, links, reminders and access you actually depend on. If someone else needs the data, have them try it with their own account.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="37" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>4. Record expected and observed behaviour, evidence and the next action. A file count or a completed download is not proof that a workflow can be recovered.</t>
+          <t>4. Mark what works, what doesn't, what you haven't checked, and what you need to fix next. A successful download by itself does not mean the export is usable.</t>
         </is>
       </c>
     </row>
@@ -852,26 +827,19 @@
     <row r="14" ht="29" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>What the current Checks sheet records</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
+          <t>What you have checked so far</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Check rows in use</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="n">
+          <t>Items in this checklist</t>
+        </is>
+      </c>
+      <c r="E15" s="8">
         <f>SUM(Checks!I11:I23)</f>
-        <v>9</v>
+        <v/>
       </c>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
@@ -880,12 +848,12 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Passes recorded with evidence</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="n">
-        <f>COUNTIF(Checks!H11:H23,"Pass recorded")</f>
-        <v>0</v>
+          <t>Items marked Works</t>
+        </is>
+      </c>
+      <c r="E16" s="8">
+        <f>COUNTIF(Checks!H11:H23,"Looks good")</f>
+        <v/>
       </c>
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
@@ -894,12 +862,12 @@
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Checks still not tested</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="n">
-        <f>COUNTIF(Checks!H11:H23,"Not tested")</f>
-        <v>9</v>
+          <t>Items not checked yet</t>
+        </is>
+      </c>
+      <c r="E17" s="8">
+        <f>COUNTIF(Checks!H11:H23,"Not checked")</f>
+        <v/>
       </c>
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
@@ -908,12 +876,12 @@
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>User exclusions with reasons</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="n">
-        <f>COUNTIF(Checks!H11:H23,"Excluded by user")</f>
-        <v>0</v>
+          <t>Items marked Doesn't apply</t>
+        </is>
+      </c>
+      <c r="E18" s="8">
+        <f>COUNTIF(Checks!H11:H23,"Doesn't apply")</f>
+        <v/>
       </c>
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
@@ -922,12 +890,12 @@
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Other follow-up or input gaps</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="n">
-        <f>SUM(Checks!I11:I23)-COUNTIF(Checks!H11:H23,"Pass recorded")-COUNTIF(Checks!H11:H23,"Not tested")-COUNTIF(Checks!H11:H23,"Excluded by user")</f>
-        <v>0</v>
+          <t>Items that still need information or a fix</t>
+        </is>
+      </c>
+      <c r="E19" s="8">
+        <f>SUM(Checks!I11:I23)-COUNTIF(Checks!H11:H23,"Looks good")-COUNTIF(Checks!H11:H23,"Not checked")-COUNTIF(Checks!H11:H23,"Doesn't apply")</f>
+        <v/>
       </c>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
@@ -936,16 +904,9 @@
     <row r="20" ht="37" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>These are counts of your entries, not a completeness, security or recovery score. A recorded pass can be wrong. An excluded check is not a passed check.</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
+          <t>These are only counts of what you entered. They do not prove that the export is complete, secure, or safe to delete.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -960,35 +921,28 @@
     <row r="22" ht="29" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>How to use the file</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
+          <t>How to use the workbook</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="39" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Blue text on pale cells is editable. The Checks sheet includes four empty rows for additional tests. Formula cells are lightly protected against accidental edits; there is no password and protection is not security.</t>
+          <t>Blue text on pale cells is where you type. The Checks sheet has extra blank rows if you need them. Formula cells are lightly protected only to prevent accidental edits.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="39" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Use the Example sheet only as a fictional illustration. Use the browser-readable REHEARSAL.md to copy the method into another tool. Nothing is automatically saved outside this workbook or sent to Eterna.</t>
+          <t>The Example sheet is fictional and only shows how the checklist can uncover a problem. Nothing is automatically uploaded or sent to Eterna.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="39" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Write descriptions and evidence locations, not passwords, recovery codes, secret links or copied sensitive records. Share the completed worksheet only with people who should see its contents.</t>
+          <t>Do not put passwords, recovery codes, secret links or copies of sensitive records in this workbook. Share the completed file only with people who should see it.</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1283,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0043161E"/>
     <outlinePr summaryBelow="1" summaryRight="0"/>
@@ -1352,16 +1306,9 @@
     <row r="1" ht="29" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Eterna Clarity | Your rehearsal</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+          <t>Eterna Clarity | Your export check</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -1376,21 +1323,14 @@
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Export and Recovery Rehearsal</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
+          <t>Export Check: Can I Still Use My Data?</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>One export, one destination, one real task. Keep the originals and test in an authorised separate location.</t>
+          <t>Check whether the files, links, access and everyday actions you actually need still work outside the old app.</t>
         </is>
       </c>
     </row>
@@ -1407,16 +1347,20 @@
     <row r="6" ht="35" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Source app / version</t>
+          <t>App or service I exported from</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr"/>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Export date and scope</t>
+          <t>Export date / what I exported</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -1431,16 +1375,20 @@
     <row r="8" ht="35" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Destination / version</t>
+          <t>Where I'm moving or storing it</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr"/>
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="18" t="n"/>
       <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Checked by / date</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="18" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -1455,42 +1403,42 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Check area</t>
+          <t>What to check</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Sample / scope</t>
+          <t>Example I checked</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Expected behaviour</t>
+          <t>What should happen</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>What actually happened</t>
+          <t>What happened</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Evidence / how checked</t>
+          <t>How I checked it</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>Your result</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Next action / exclusion reason</t>
+          <t>What I'll do next / why it doesn't apply</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>Record check</t>
+          <t>Quick check</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1502,7 +1450,7 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Readable content</t>
+          <t>Files or records I can open</t>
         </is>
       </c>
       <c r="B11" s="14" t="n"/>
@@ -1511,23 +1459,23 @@
       <c r="E11" s="14" t="n"/>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G11" s="14" t="n"/>
-      <c r="H11" s="15" t="str">
-        <f>IF(LEN(TRIM(A11&amp;B11&amp;C11&amp;D11&amp;E11&amp;F11&amp;G11))=0,"",IF(LEN(TRIM(A11))=0,"Name the check",IF(F11="Not applicable",IF(LEN(TRIM(G11))&gt;0,"Excluded by user","Explain exclusion"),IF(F11="Pass",IF(AND(LEN(TRIM(B11))&gt;0,LEN(TRIM(C11))&gt;0,LEN(TRIM(D11))&gt;0,LEN(TRIM(E11))&gt;0),"Pass recorded","Evidence missing"),IF(F11="Fail",IF(LEN(TRIM(G11))&gt;0,"Follow up","Add next action"),IF(OR(F11="",F11="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I11" s="16" t="n">
+      <c r="H11" s="15">
+        <f>IF(LEN(TRIM(A11&amp;B11&amp;C11&amp;D11&amp;E11&amp;F11&amp;G11))=0,"",IF(LEN(TRIM(A11))=0,"Name what you are checking",IF(F11="Doesn't apply",IF(LEN(TRIM(G11))&gt;0,"Doesn't apply","Say why"),IF(F11="Works",IF(AND(LEN(TRIM(B11))&gt;0,LEN(TRIM(C11))&gt;0,LEN(TRIM(D11))&gt;0,LEN(TRIM(E11))&gt;0),"Looks good","Add how you checked it"),IF(F11="Doesn't work",IF(LEN(TRIM(G11))&gt;0,"Needs fixing","Add next step"),IF(OR(F11="",F11="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I11" s="16">
         <f>IF(H11="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Attachments</t>
+          <t>Attachments or images</t>
         </is>
       </c>
       <c r="B12" s="14" t="n"/>
@@ -1536,23 +1484,23 @@
       <c r="E12" s="14" t="n"/>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G12" s="14" t="n"/>
-      <c r="H12" s="15" t="str">
-        <f>IF(LEN(TRIM(A12&amp;B12&amp;C12&amp;D12&amp;E12&amp;F12&amp;G12))=0,"",IF(LEN(TRIM(A12))=0,"Name the check",IF(F12="Not applicable",IF(LEN(TRIM(G12))&gt;0,"Excluded by user","Explain exclusion"),IF(F12="Pass",IF(AND(LEN(TRIM(B12))&gt;0,LEN(TRIM(C12))&gt;0,LEN(TRIM(D12))&gt;0,LEN(TRIM(E12))&gt;0),"Pass recorded","Evidence missing"),IF(F12="Fail",IF(LEN(TRIM(G12))&gt;0,"Follow up","Add next action"),IF(OR(F12="",F12="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I12" s="16" t="n">
+      <c r="H12" s="15">
+        <f>IF(LEN(TRIM(A12&amp;B12&amp;C12&amp;D12&amp;E12&amp;F12&amp;G12))=0,"",IF(LEN(TRIM(A12))=0,"Name what you are checking",IF(F12="Doesn't apply",IF(LEN(TRIM(G12))&gt;0,"Doesn't apply","Say why"),IF(F12="Works",IF(AND(LEN(TRIM(B12))&gt;0,LEN(TRIM(C12))&gt;0,LEN(TRIM(D12))&gt;0,LEN(TRIM(E12))&gt;0),"Looks good","Add how you checked it"),IF(F12="Doesn't work",IF(LEN(TRIM(G12))&gt;0,"Needs fixing","Add next step"),IF(OR(F12="",F12="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I12" s="16">
         <f>IF(H12="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Links and relationships</t>
+          <t>Links between items</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
@@ -1561,23 +1509,23 @@
       <c r="E13" s="14" t="n"/>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G13" s="14" t="n"/>
-      <c r="H13" s="15" t="str">
-        <f>IF(LEN(TRIM(A13&amp;B13&amp;C13&amp;D13&amp;E13&amp;F13&amp;G13))=0,"",IF(LEN(TRIM(A13))=0,"Name the check",IF(F13="Not applicable",IF(LEN(TRIM(G13))&gt;0,"Excluded by user","Explain exclusion"),IF(F13="Pass",IF(AND(LEN(TRIM(B13))&gt;0,LEN(TRIM(C13))&gt;0,LEN(TRIM(D13))&gt;0,LEN(TRIM(E13))&gt;0),"Pass recorded","Evidence missing"),IF(F13="Fail",IF(LEN(TRIM(G13))&gt;0,"Follow up","Add next action"),IF(OR(F13="",F13="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I13" s="16" t="n">
+      <c r="H13" s="15">
+        <f>IF(LEN(TRIM(A13&amp;B13&amp;C13&amp;D13&amp;E13&amp;F13&amp;G13))=0,"",IF(LEN(TRIM(A13))=0,"Name what you are checking",IF(F13="Doesn't apply",IF(LEN(TRIM(G13))&gt;0,"Doesn't apply","Say why"),IF(F13="Works",IF(AND(LEN(TRIM(B13))&gt;0,LEN(TRIM(C13))&gt;0,LEN(TRIM(D13))&gt;0,LEN(TRIM(E13))&gt;0),"Looks good","Add how you checked it"),IF(F13="Doesn't work",IF(LEN(TRIM(G13))&gt;0,"Needs fixing","Add next step"),IF(OR(F13="",F13="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I13" s="16">
         <f>IF(H13="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Comments and history</t>
+          <t>History or comments</t>
         </is>
       </c>
       <c r="B14" s="14" t="n"/>
@@ -1586,23 +1534,23 @@
       <c r="E14" s="14" t="n"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G14" s="14" t="n"/>
-      <c r="H14" s="15" t="str">
-        <f>IF(LEN(TRIM(A14&amp;B14&amp;C14&amp;D14&amp;E14&amp;F14&amp;G14))=0,"",IF(LEN(TRIM(A14))=0,"Name the check",IF(F14="Not applicable",IF(LEN(TRIM(G14))&gt;0,"Excluded by user","Explain exclusion"),IF(F14="Pass",IF(AND(LEN(TRIM(B14))&gt;0,LEN(TRIM(C14))&gt;0,LEN(TRIM(D14))&gt;0,LEN(TRIM(E14))&gt;0),"Pass recorded","Evidence missing"),IF(F14="Fail",IF(LEN(TRIM(G14))&gt;0,"Follow up","Add next action"),IF(OR(F14="",F14="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I14" s="16" t="n">
+      <c r="H14" s="15">
+        <f>IF(LEN(TRIM(A14&amp;B14&amp;C14&amp;D14&amp;E14&amp;F14&amp;G14))=0,"",IF(LEN(TRIM(A14))=0,"Name what you are checking",IF(F14="Doesn't apply",IF(LEN(TRIM(G14))&gt;0,"Doesn't apply","Say why"),IF(F14="Works",IF(AND(LEN(TRIM(B14))&gt;0,LEN(TRIM(C14))&gt;0,LEN(TRIM(D14))&gt;0,LEN(TRIM(E14))&gt;0),"Looks good","Add how you checked it"),IF(F14="Doesn't work",IF(LEN(TRIM(G14))&gt;0,"Needs fixing","Add next step"),IF(OR(F14="",F14="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I14" s="16">
         <f>IF(H14="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Views and calculations</t>
+          <t>Views, filters or calculations</t>
         </is>
       </c>
       <c r="B15" s="14" t="n"/>
@@ -1611,23 +1559,23 @@
       <c r="E15" s="14" t="n"/>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G15" s="14" t="n"/>
-      <c r="H15" s="15" t="str">
-        <f>IF(LEN(TRIM(A15&amp;B15&amp;C15&amp;D15&amp;E15&amp;F15&amp;G15))=0,"",IF(LEN(TRIM(A15))=0,"Name the check",IF(F15="Not applicable",IF(LEN(TRIM(G15))&gt;0,"Excluded by user","Explain exclusion"),IF(F15="Pass",IF(AND(LEN(TRIM(B15))&gt;0,LEN(TRIM(C15))&gt;0,LEN(TRIM(D15))&gt;0,LEN(TRIM(E15))&gt;0),"Pass recorded","Evidence missing"),IF(F15="Fail",IF(LEN(TRIM(G15))&gt;0,"Follow up","Add next action"),IF(OR(F15="",F15="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I15" s="16" t="n">
+      <c r="H15" s="15">
+        <f>IF(LEN(TRIM(A15&amp;B15&amp;C15&amp;D15&amp;E15&amp;F15&amp;G15))=0,"",IF(LEN(TRIM(A15))=0,"Name what you are checking",IF(F15="Doesn't apply",IF(LEN(TRIM(G15))&gt;0,"Doesn't apply","Say why"),IF(F15="Works",IF(AND(LEN(TRIM(B15))&gt;0,LEN(TRIM(C15))&gt;0,LEN(TRIM(D15))&gt;0,LEN(TRIM(E15))&gt;0),"Looks good","Add how you checked it"),IF(F15="Doesn't work",IF(LEN(TRIM(G15))&gt;0,"Needs fixing","Add next step"),IF(OR(F15="",F15="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I15" s="16">
         <f>IF(H15="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Reminders and automations</t>
+          <t>Reminders or automatic actions</t>
         </is>
       </c>
       <c r="B16" s="14" t="n"/>
@@ -1636,23 +1584,23 @@
       <c r="E16" s="14" t="n"/>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G16" s="14" t="n"/>
-      <c r="H16" s="15" t="str">
-        <f>IF(LEN(TRIM(A16&amp;B16&amp;C16&amp;D16&amp;E16&amp;F16&amp;G16))=0,"",IF(LEN(TRIM(A16))=0,"Name the check",IF(F16="Not applicable",IF(LEN(TRIM(G16))&gt;0,"Excluded by user","Explain exclusion"),IF(F16="Pass",IF(AND(LEN(TRIM(B16))&gt;0,LEN(TRIM(C16))&gt;0,LEN(TRIM(D16))&gt;0,LEN(TRIM(E16))&gt;0),"Pass recorded","Evidence missing"),IF(F16="Fail",IF(LEN(TRIM(G16))&gt;0,"Follow up","Add next action"),IF(OR(F16="",F16="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I16" s="16" t="n">
+      <c r="H16" s="15">
+        <f>IF(LEN(TRIM(A16&amp;B16&amp;C16&amp;D16&amp;E16&amp;F16&amp;G16))=0,"",IF(LEN(TRIM(A16))=0,"Name what you are checking",IF(F16="Doesn't apply",IF(LEN(TRIM(G16))&gt;0,"Doesn't apply","Say why"),IF(F16="Works",IF(AND(LEN(TRIM(B16))&gt;0,LEN(TRIM(C16))&gt;0,LEN(TRIM(D16))&gt;0,LEN(TRIM(E16))&gt;0),"Looks good","Add how you checked it"),IF(F16="Doesn't work",IF(LEN(TRIM(G16))&gt;0,"Needs fixing","Add next step"),IF(OR(F16="",F16="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I16" s="16">
         <f>IF(H16="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Access and ownership</t>
+          <t>Other people's access</t>
         </is>
       </c>
       <c r="B17" s="14" t="n"/>
@@ -1661,23 +1609,23 @@
       <c r="E17" s="14" t="n"/>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G17" s="14" t="n"/>
-      <c r="H17" s="15" t="str">
-        <f>IF(LEN(TRIM(A17&amp;B17&amp;C17&amp;D17&amp;E17&amp;F17&amp;G17))=0,"",IF(LEN(TRIM(A17))=0,"Name the check",IF(F17="Not applicable",IF(LEN(TRIM(G17))&gt;0,"Excluded by user","Explain exclusion"),IF(F17="Pass",IF(AND(LEN(TRIM(B17))&gt;0,LEN(TRIM(C17))&gt;0,LEN(TRIM(D17))&gt;0,LEN(TRIM(E17))&gt;0),"Pass recorded","Evidence missing"),IF(F17="Fail",IF(LEN(TRIM(G17))&gt;0,"Follow up","Add next action"),IF(OR(F17="",F17="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I17" s="16" t="n">
+      <c r="H17" s="15">
+        <f>IF(LEN(TRIM(A17&amp;B17&amp;C17&amp;D17&amp;E17&amp;F17&amp;G17))=0,"",IF(LEN(TRIM(A17))=0,"Name what you are checking",IF(F17="Doesn't apply",IF(LEN(TRIM(G17))&gt;0,"Doesn't apply","Say why"),IF(F17="Works",IF(AND(LEN(TRIM(B17))&gt;0,LEN(TRIM(C17))&gt;0,LEN(TRIM(D17))&gt;0,LEN(TRIM(E17))&gt;0),"Looks good","Add how you checked it"),IF(F17="Doesn't work",IF(LEN(TRIM(G17))&gt;0,"Needs fixing","Add next step"),IF(OR(F17="",F17="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I17" s="16">
         <f>IF(H17="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>Scope and exceptions</t>
+          <t>Missing or skipped items</t>
         </is>
       </c>
       <c r="B18" s="14" t="n"/>
@@ -1686,23 +1634,23 @@
       <c r="E18" s="14" t="n"/>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G18" s="14" t="n"/>
-      <c r="H18" s="15" t="str">
-        <f>IF(LEN(TRIM(A18&amp;B18&amp;C18&amp;D18&amp;E18&amp;F18&amp;G18))=0,"",IF(LEN(TRIM(A18))=0,"Name the check",IF(F18="Not applicable",IF(LEN(TRIM(G18))&gt;0,"Excluded by user","Explain exclusion"),IF(F18="Pass",IF(AND(LEN(TRIM(B18))&gt;0,LEN(TRIM(C18))&gt;0,LEN(TRIM(D18))&gt;0,LEN(TRIM(E18))&gt;0),"Pass recorded","Evidence missing"),IF(F18="Fail",IF(LEN(TRIM(G18))&gt;0,"Follow up","Add next action"),IF(OR(F18="",F18="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I18" s="16" t="n">
+      <c r="H18" s="15">
+        <f>IF(LEN(TRIM(A18&amp;B18&amp;C18&amp;D18&amp;E18&amp;F18&amp;G18))=0,"",IF(LEN(TRIM(A18))=0,"Name what you are checking",IF(F18="Doesn't apply",IF(LEN(TRIM(G18))&gt;0,"Doesn't apply","Say why"),IF(F18="Works",IF(AND(LEN(TRIM(B18))&gt;0,LEN(TRIM(C18))&gt;0,LEN(TRIM(D18))&gt;0,LEN(TRIM(E18))&gt;0),"Looks good","Add how you checked it"),IF(F18="Doesn't work",IF(LEN(TRIM(G18))&gt;0,"Needs fixing","Add next step"),IF(OR(F18="",F18="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I18" s="16">
         <f>IF(H18="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>One real next action</t>
+          <t>One real thing I need to do</t>
         </is>
       </c>
       <c r="B19" s="14" t="n"/>
@@ -1711,17 +1659,17 @@
       <c r="E19" s="14" t="n"/>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G19" s="14" t="n"/>
-      <c r="H19" s="15" t="str">
-        <f>IF(LEN(TRIM(A19&amp;B19&amp;C19&amp;D19&amp;E19&amp;F19&amp;G19))=0,"",IF(LEN(TRIM(A19))=0,"Name the check",IF(F19="Not applicable",IF(LEN(TRIM(G19))&gt;0,"Excluded by user","Explain exclusion"),IF(F19="Pass",IF(AND(LEN(TRIM(B19))&gt;0,LEN(TRIM(C19))&gt;0,LEN(TRIM(D19))&gt;0,LEN(TRIM(E19))&gt;0),"Pass recorded","Evidence missing"),IF(F19="Fail",IF(LEN(TRIM(G19))&gt;0,"Follow up","Add next action"),IF(OR(F19="",F19="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I19" s="16" t="n">
+      <c r="H19" s="15">
+        <f>IF(LEN(TRIM(A19&amp;B19&amp;C19&amp;D19&amp;E19&amp;F19&amp;G19))=0,"",IF(LEN(TRIM(A19))=0,"Name what you are checking",IF(F19="Doesn't apply",IF(LEN(TRIM(G19))&gt;0,"Doesn't apply","Say why"),IF(F19="Works",IF(AND(LEN(TRIM(B19))&gt;0,LEN(TRIM(C19))&gt;0,LEN(TRIM(D19))&gt;0,LEN(TRIM(E19))&gt;0),"Looks good","Add how you checked it"),IF(F19="Doesn't work",IF(LEN(TRIM(G19))&gt;0,"Needs fixing","Add next step"),IF(OR(F19="",F19="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I19" s="16">
         <f>IF(H19="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="20" ht="90" customHeight="1">
@@ -1730,15 +1678,19 @@
       <c r="C20" s="14" t="n"/>
       <c r="D20" s="14" t="n"/>
       <c r="E20" s="14" t="n"/>
-      <c r="F20" s="14" t="n"/>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
       <c r="G20" s="14" t="n"/>
-      <c r="H20" s="15" t="str">
-        <f>IF(LEN(TRIM(A20&amp;B20&amp;C20&amp;D20&amp;E20&amp;F20&amp;G20))=0,"",IF(LEN(TRIM(A20))=0,"Name the check",IF(F20="Not applicable",IF(LEN(TRIM(G20))&gt;0,"Excluded by user","Explain exclusion"),IF(F20="Pass",IF(AND(LEN(TRIM(B20))&gt;0,LEN(TRIM(C20))&gt;0,LEN(TRIM(D20))&gt;0,LEN(TRIM(E20))&gt;0),"Pass recorded","Evidence missing"),IF(F20="Fail",IF(LEN(TRIM(G20))&gt;0,"Follow up","Add next action"),IF(OR(F20="",F20="Not tested"),"Not tested","Check status"))))))</f>
-        <v/>
-      </c>
-      <c r="I20" s="16" t="n">
+      <c r="H20" s="15">
+        <f>IF(LEN(TRIM(A20&amp;B20&amp;C20&amp;D20&amp;E20&amp;F20&amp;G20))=0,"",IF(LEN(TRIM(A20))=0,"Name what you are checking",IF(F20="Doesn't apply",IF(LEN(TRIM(G20))&gt;0,"Doesn't apply","Say why"),IF(F20="Works",IF(AND(LEN(TRIM(B20))&gt;0,LEN(TRIM(C20))&gt;0,LEN(TRIM(D20))&gt;0,LEN(TRIM(E20))&gt;0),"Looks good","Add how you checked it"),IF(F20="Doesn't work",IF(LEN(TRIM(G20))&gt;0,"Needs fixing","Add next step"),IF(OR(F20="",F20="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I20" s="16">
         <f>IF(H20="",0,1)</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="21" ht="90" customHeight="1">
@@ -1747,15 +1699,19 @@
       <c r="C21" s="14" t="n"/>
       <c r="D21" s="14" t="n"/>
       <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="n"/>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
       <c r="G21" s="14" t="n"/>
-      <c r="H21" s="15" t="str">
-        <f>IF(LEN(TRIM(A21&amp;B21&amp;C21&amp;D21&amp;E21&amp;F21&amp;G21))=0,"",IF(LEN(TRIM(A21))=0,"Name the check",IF(F21="Not applicable",IF(LEN(TRIM(G21))&gt;0,"Excluded by user","Explain exclusion"),IF(F21="Pass",IF(AND(LEN(TRIM(B21))&gt;0,LEN(TRIM(C21))&gt;0,LEN(TRIM(D21))&gt;0,LEN(TRIM(E21))&gt;0),"Pass recorded","Evidence missing"),IF(F21="Fail",IF(LEN(TRIM(G21))&gt;0,"Follow up","Add next action"),IF(OR(F21="",F21="Not tested"),"Not tested","Check status"))))))</f>
-        <v/>
-      </c>
-      <c r="I21" s="16" t="n">
+      <c r="H21" s="15">
+        <f>IF(LEN(TRIM(A21&amp;B21&amp;C21&amp;D21&amp;E21&amp;F21&amp;G21))=0,"",IF(LEN(TRIM(A21))=0,"Name what you are checking",IF(F21="Doesn't apply",IF(LEN(TRIM(G21))&gt;0,"Doesn't apply","Say why"),IF(F21="Works",IF(AND(LEN(TRIM(B21))&gt;0,LEN(TRIM(C21))&gt;0,LEN(TRIM(D21))&gt;0,LEN(TRIM(E21))&gt;0),"Looks good","Add how you checked it"),IF(F21="Doesn't work",IF(LEN(TRIM(G21))&gt;0,"Needs fixing","Add next step"),IF(OR(F21="",F21="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I21" s="16">
         <f>IF(H21="",0,1)</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="22" ht="90" customHeight="1">
@@ -1764,15 +1720,19 @@
       <c r="C22" s="14" t="n"/>
       <c r="D22" s="14" t="n"/>
       <c r="E22" s="14" t="n"/>
-      <c r="F22" s="14" t="n"/>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
       <c r="G22" s="14" t="n"/>
-      <c r="H22" s="15" t="str">
-        <f>IF(LEN(TRIM(A22&amp;B22&amp;C22&amp;D22&amp;E22&amp;F22&amp;G22))=0,"",IF(LEN(TRIM(A22))=0,"Name the check",IF(F22="Not applicable",IF(LEN(TRIM(G22))&gt;0,"Excluded by user","Explain exclusion"),IF(F22="Pass",IF(AND(LEN(TRIM(B22))&gt;0,LEN(TRIM(C22))&gt;0,LEN(TRIM(D22))&gt;0,LEN(TRIM(E22))&gt;0),"Pass recorded","Evidence missing"),IF(F22="Fail",IF(LEN(TRIM(G22))&gt;0,"Follow up","Add next action"),IF(OR(F22="",F22="Not tested"),"Not tested","Check status"))))))</f>
-        <v/>
-      </c>
-      <c r="I22" s="16" t="n">
+      <c r="H22" s="15">
+        <f>IF(LEN(TRIM(A22&amp;B22&amp;C22&amp;D22&amp;E22&amp;F22&amp;G22))=0,"",IF(LEN(TRIM(A22))=0,"Name what you are checking",IF(F22="Doesn't apply",IF(LEN(TRIM(G22))&gt;0,"Doesn't apply","Say why"),IF(F22="Works",IF(AND(LEN(TRIM(B22))&gt;0,LEN(TRIM(C22))&gt;0,LEN(TRIM(D22))&gt;0,LEN(TRIM(E22))&gt;0),"Looks good","Add how you checked it"),IF(F22="Doesn't work",IF(LEN(TRIM(G22))&gt;0,"Needs fixing","Add next step"),IF(OR(F22="",F22="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I22" s="16">
         <f>IF(H22="",0,1)</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="23" ht="90" customHeight="1">
@@ -1781,15 +1741,19 @@
       <c r="C23" s="14" t="n"/>
       <c r="D23" s="14" t="n"/>
       <c r="E23" s="14" t="n"/>
-      <c r="F23" s="14" t="n"/>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
       <c r="G23" s="14" t="n"/>
-      <c r="H23" s="15" t="str">
-        <f>IF(LEN(TRIM(A23&amp;B23&amp;C23&amp;D23&amp;E23&amp;F23&amp;G23))=0,"",IF(LEN(TRIM(A23))=0,"Name the check",IF(F23="Not applicable",IF(LEN(TRIM(G23))&gt;0,"Excluded by user","Explain exclusion"),IF(F23="Pass",IF(AND(LEN(TRIM(B23))&gt;0,LEN(TRIM(C23))&gt;0,LEN(TRIM(D23))&gt;0,LEN(TRIM(E23))&gt;0),"Pass recorded","Evidence missing"),IF(F23="Fail",IF(LEN(TRIM(G23))&gt;0,"Follow up","Add next action"),IF(OR(F23="",F23="Not tested"),"Not tested","Check status"))))))</f>
-        <v/>
-      </c>
-      <c r="I23" s="16" t="n">
+      <c r="H23" s="15">
+        <f>IF(LEN(TRIM(A23&amp;B23&amp;C23&amp;D23&amp;E23&amp;F23&amp;G23))=0,"",IF(LEN(TRIM(A23))=0,"Name what you are checking",IF(F23="Doesn't apply",IF(LEN(TRIM(G23))&gt;0,"Doesn't apply","Say why"),IF(F23="Works",IF(AND(LEN(TRIM(B23))&gt;0,LEN(TRIM(C23))&gt;0,LEN(TRIM(D23))&gt;0,LEN(TRIM(E23))&gt;0),"Looks good","Add how you checked it"),IF(F23="Doesn't work",IF(LEN(TRIM(G23))&gt;0,"Needs fixing","Add next step"),IF(OR(F23="",F23="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I23" s="16">
         <f>IF(H23="",0,1)</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1805,16 +1769,9 @@
     <row r="25" ht="35" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>A recorded pass is your observation, not automatic verification. Test permissions using the intended receiver. Do not paste credentials or sensitive source records. Four blank rows allow additional checks.</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
+          <t>A result is what you observed in this check, not a guarantee. If someone else needs the export, have them try it with their own access. Do not put passwords or sensitive records here.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -2145,7 +2102,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="F11:F23" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Choose a listed result" error="Use Not tested, Pass, Fail or Not applicable." promptTitle="Record only what you checked" prompt="Pass needs a sample, expected and actual behaviour, plus evidence. An exclusion needs a reason." type="list" errorStyle="stop">
-      <formula1>"Not tested,Pass,Fail,Not applicable"</formula1>
+      <formula1>"Not checked,Works,Doesn't work,Doesn't apply"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>
@@ -2158,12 +2115,12 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <legacyDrawing ns1:id="anysvml"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0043161E"/>
     <outlinePr summaryBelow="1" summaryRight="0"/>
@@ -2189,13 +2146,6 @@
           <t>Eterna Clarity | Fictional example</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -2210,21 +2160,14 @@
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Export and Recovery Rehearsal</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
+          <t>Export Check: Can I Still Use My Data?</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Fictional club workspace. These outcomes are invented to illustrate the method, not claims about an actual product.</t>
+          <t>Fictional example: a community club moves its equipment notes and finds several things that still depend on the old app.</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2184,7 @@
     <row r="6" ht="35" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Source app / version</t>
+          <t>App or service I exported from</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -2249,9 +2192,11 @@
           <t>Fictional club workspace</t>
         </is>
       </c>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Export date and scope</t>
+          <t>Export date / what I exported</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
@@ -2259,6 +2204,8 @@
           <t>16 Sep 2026; selected notes and tasks only</t>
         </is>
       </c>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -2273,7 +2220,7 @@
     <row r="8" ht="35" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Destination / version</t>
+          <t>Where I'm moving or storing it</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -2281,6 +2228,8 @@
           <t>Separate test folder and task list</t>
         </is>
       </c>
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="18" t="n"/>
       <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Checked by / date</t>
@@ -2291,6 +2240,8 @@
           <t>Fictional replacement coordinator; 16 Sep 2026</t>
         </is>
       </c>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="18" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -2305,42 +2256,42 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Check area</t>
+          <t>What to check</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Sample / scope</t>
+          <t>Example I checked</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Expected behaviour</t>
+          <t>What should happen</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>What actually happened</t>
+          <t>What happened</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Evidence / how checked</t>
+          <t>How I checked it</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>Your result</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Next action / exclusion reason</t>
+          <t>What I'll do next / why it doesn't apply</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>Record check</t>
+          <t>Quick check</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2352,7 +2303,7 @@
     <row r="11" ht="102" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Readable content</t>
+          <t>Files or records I can open</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -2367,7 +2318,7 @@
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>Text opens in the destination folder</t>
+          <t>Text opens in the new folder</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -2377,23 +2328,23 @@
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Works</t>
         </is>
       </c>
       <c r="G11" s="14" t="inlineStr"/>
-      <c r="H11" s="15" t="str">
-        <f>IF(LEN(TRIM(A11&amp;B11&amp;C11&amp;D11&amp;E11&amp;F11&amp;G11))=0,"",IF(LEN(TRIM(A11))=0,"Name the check",IF(F11="Not applicable",IF(LEN(TRIM(G11))&gt;0,"Excluded by user","Explain exclusion"),IF(F11="Pass",IF(AND(LEN(TRIM(B11))&gt;0,LEN(TRIM(C11))&gt;0,LEN(TRIM(D11))&gt;0,LEN(TRIM(E11))&gt;0),"Pass recorded","Evidence missing"),IF(F11="Fail",IF(LEN(TRIM(G11))&gt;0,"Follow up","Add next action"),IF(OR(F11="",F11="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Pass recorded</v>
-      </c>
-      <c r="I11" s="16" t="n">
+      <c r="H11" s="15">
+        <f>IF(LEN(TRIM(A11&amp;B11&amp;C11&amp;D11&amp;E11&amp;F11&amp;G11))=0,"",IF(LEN(TRIM(A11))=0,"Name what you are checking",IF(F11="Doesn't apply",IF(LEN(TRIM(G11))&gt;0,"Doesn't apply","Say why"),IF(F11="Works",IF(AND(LEN(TRIM(B11))&gt;0,LEN(TRIM(C11))&gt;0,LEN(TRIM(D11))&gt;0,LEN(TRIM(E11))&gt;0),"Looks good","Add how you checked it"),IF(F11="Doesn't work",IF(LEN(TRIM(G11))&gt;0,"Needs fixing","Add next step"),IF(OR(F11="",F11="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I11" s="16">
         <f>IF(H11="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="12" ht="102" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Attachments</t>
+          <t>Attachments or images</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -2418,7 +2369,7 @@
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Doesn't work</t>
         </is>
       </c>
       <c r="G12" s="14" t="inlineStr">
@@ -2426,19 +2377,19 @@
           <t>Download the actual photo through the authorised source, then retest.</t>
         </is>
       </c>
-      <c r="H12" s="15" t="str">
-        <f>IF(LEN(TRIM(A12&amp;B12&amp;C12&amp;D12&amp;E12&amp;F12&amp;G12))=0,"",IF(LEN(TRIM(A12))=0,"Name the check",IF(F12="Not applicable",IF(LEN(TRIM(G12))&gt;0,"Excluded by user","Explain exclusion"),IF(F12="Pass",IF(AND(LEN(TRIM(B12))&gt;0,LEN(TRIM(C12))&gt;0,LEN(TRIM(D12))&gt;0,LEN(TRIM(E12))&gt;0),"Pass recorded","Evidence missing"),IF(F12="Fail",IF(LEN(TRIM(G12))&gt;0,"Follow up","Add next action"),IF(OR(F12="",F12="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Follow up</v>
-      </c>
-      <c r="I12" s="16" t="n">
+      <c r="H12" s="15">
+        <f>IF(LEN(TRIM(A12&amp;B12&amp;C12&amp;D12&amp;E12&amp;F12&amp;G12))=0,"",IF(LEN(TRIM(A12))=0,"Name what you are checking",IF(F12="Doesn't apply",IF(LEN(TRIM(G12))&gt;0,"Doesn't apply","Say why"),IF(F12="Works",IF(AND(LEN(TRIM(B12))&gt;0,LEN(TRIM(C12))&gt;0,LEN(TRIM(D12))&gt;0,LEN(TRIM(E12))&gt;0),"Looks good","Add how you checked it"),IF(F12="Doesn't work",IF(LEN(TRIM(G12))&gt;0,"Needs fixing","Add next step"),IF(OR(F12="",F12="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I12" s="16">
         <f>IF(H12="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="13" ht="102" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Links and relationships</t>
+          <t>Links between items</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -2463,27 +2414,27 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Doesn't work</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>Add a destination reference; test the link in the new location.</t>
-        </is>
-      </c>
-      <c r="H13" s="15" t="str">
-        <f>IF(LEN(TRIM(A13&amp;B13&amp;C13&amp;D13&amp;E13&amp;F13&amp;G13))=0,"",IF(LEN(TRIM(A13))=0,"Name the check",IF(F13="Not applicable",IF(LEN(TRIM(G13))&gt;0,"Excluded by user","Explain exclusion"),IF(F13="Pass",IF(AND(LEN(TRIM(B13))&gt;0,LEN(TRIM(C13))&gt;0,LEN(TRIM(D13))&gt;0,LEN(TRIM(E13))&gt;0),"Pass recorded","Evidence missing"),IF(F13="Fail",IF(LEN(TRIM(G13))&gt;0,"Follow up","Add next action"),IF(OR(F13="",F13="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Follow up</v>
-      </c>
-      <c r="I13" s="16" t="n">
+          <t>Update the link to the new copy, then test it again.</t>
+        </is>
+      </c>
+      <c r="H13" s="15">
+        <f>IF(LEN(TRIM(A13&amp;B13&amp;C13&amp;D13&amp;E13&amp;F13&amp;G13))=0,"",IF(LEN(TRIM(A13))=0,"Name what you are checking",IF(F13="Doesn't apply",IF(LEN(TRIM(G13))&gt;0,"Doesn't apply","Say why"),IF(F13="Works",IF(AND(LEN(TRIM(B13))&gt;0,LEN(TRIM(C13))&gt;0,LEN(TRIM(D13))&gt;0,LEN(TRIM(E13))&gt;0),"Looks good","Add how you checked it"),IF(F13="Doesn't work",IF(LEN(TRIM(G13))&gt;0,"Needs fixing","Add next step"),IF(OR(F13="",F13="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I13" s="16">
         <f>IF(H13="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="14" ht="102" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Comments and history</t>
+          <t>History or comments</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -2496,7 +2447,7 @@
       <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Doesn't apply</t>
         </is>
       </c>
       <c r="G14" s="14" t="inlineStr">
@@ -2504,19 +2455,19 @@
           <t>Only the current approved note is needed. Original history is retained separately.</t>
         </is>
       </c>
-      <c r="H14" s="15" t="str">
-        <f>IF(LEN(TRIM(A14&amp;B14&amp;C14&amp;D14&amp;E14&amp;F14&amp;G14))=0,"",IF(LEN(TRIM(A14))=0,"Name the check",IF(F14="Not applicable",IF(LEN(TRIM(G14))&gt;0,"Excluded by user","Explain exclusion"),IF(F14="Pass",IF(AND(LEN(TRIM(B14))&gt;0,LEN(TRIM(C14))&gt;0,LEN(TRIM(D14))&gt;0,LEN(TRIM(E14))&gt;0),"Pass recorded","Evidence missing"),IF(F14="Fail",IF(LEN(TRIM(G14))&gt;0,"Follow up","Add next action"),IF(OR(F14="",F14="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Excluded by user</v>
-      </c>
-      <c r="I14" s="16" t="n">
+      <c r="H14" s="15">
+        <f>IF(LEN(TRIM(A14&amp;B14&amp;C14&amp;D14&amp;E14&amp;F14&amp;G14))=0,"",IF(LEN(TRIM(A14))=0,"Name what you are checking",IF(F14="Doesn't apply",IF(LEN(TRIM(G14))&gt;0,"Doesn't apply","Say why"),IF(F14="Works",IF(AND(LEN(TRIM(B14))&gt;0,LEN(TRIM(C14))&gt;0,LEN(TRIM(D14))&gt;0,LEN(TRIM(E14))&gt;0),"Looks good","Add how you checked it"),IF(F14="Doesn't work",IF(LEN(TRIM(G14))&gt;0,"Needs fixing","Add next step"),IF(OR(F14="",F14="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I14" s="16">
         <f>IF(H14="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="15" ht="102" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Views and calculations</t>
+          <t>Views, filters or calculations</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2533,27 +2484,27 @@
       <c r="E15" s="14" t="inlineStr"/>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>Test the destination filter; a list export does not prove the filter survived.</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="str">
-        <f>IF(LEN(TRIM(A15&amp;B15&amp;C15&amp;D15&amp;E15&amp;F15&amp;G15))=0,"",IF(LEN(TRIM(A15))=0,"Name the check",IF(F15="Not applicable",IF(LEN(TRIM(G15))&gt;0,"Excluded by user","Explain exclusion"),IF(F15="Pass",IF(AND(LEN(TRIM(B15))&gt;0,LEN(TRIM(C15))&gt;0,LEN(TRIM(D15))&gt;0,LEN(TRIM(E15))&gt;0),"Pass recorded","Evidence missing"),IF(F15="Fail",IF(LEN(TRIM(G15))&gt;0,"Follow up","Add next action"),IF(OR(F15="",F15="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I15" s="16" t="n">
+          <t>Test the filter in the new app or file; a list export does not prove the filter still works.</t>
+        </is>
+      </c>
+      <c r="H15" s="15">
+        <f>IF(LEN(TRIM(A15&amp;B15&amp;C15&amp;D15&amp;E15&amp;F15&amp;G15))=0,"",IF(LEN(TRIM(A15))=0,"Name what you are checking",IF(F15="Doesn't apply",IF(LEN(TRIM(G15))&gt;0,"Doesn't apply","Say why"),IF(F15="Works",IF(AND(LEN(TRIM(B15))&gt;0,LEN(TRIM(C15))&gt;0,LEN(TRIM(D15))&gt;0,LEN(TRIM(E15))&gt;0),"Looks good","Add how you checked it"),IF(F15="Doesn't work",IF(LEN(TRIM(G15))&gt;0,"Needs fixing","Add next step"),IF(OR(F15="",F15="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I15" s="16">
         <f>IF(H15="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="16" ht="102" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Reminders and automations</t>
+          <t>Reminders or automatic actions</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -2563,14 +2514,14 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Receive a reminder in the destination</t>
+          <t>Receive a reminder in the new app</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr"/>
       <c r="E16" s="14" t="inlineStr"/>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="G16" s="14" t="inlineStr">
@@ -2578,29 +2529,29 @@
           <t>Recreate an approved reminder and test it without waiting for a real deadline.</t>
         </is>
       </c>
-      <c r="H16" s="15" t="str">
-        <f>IF(LEN(TRIM(A16&amp;B16&amp;C16&amp;D16&amp;E16&amp;F16&amp;G16))=0,"",IF(LEN(TRIM(A16))=0,"Name the check",IF(F16="Not applicable",IF(LEN(TRIM(G16))&gt;0,"Excluded by user","Explain exclusion"),IF(F16="Pass",IF(AND(LEN(TRIM(B16))&gt;0,LEN(TRIM(C16))&gt;0,LEN(TRIM(D16))&gt;0,LEN(TRIM(E16))&gt;0),"Pass recorded","Evidence missing"),IF(F16="Fail",IF(LEN(TRIM(G16))&gt;0,"Follow up","Add next action"),IF(OR(F16="",F16="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Not tested</v>
-      </c>
-      <c r="I16" s="16" t="n">
+      <c r="H16" s="15">
+        <f>IF(LEN(TRIM(A16&amp;B16&amp;C16&amp;D16&amp;E16&amp;F16&amp;G16))=0,"",IF(LEN(TRIM(A16))=0,"Name what you are checking",IF(F16="Doesn't apply",IF(LEN(TRIM(G16))&gt;0,"Doesn't apply","Say why"),IF(F16="Works",IF(AND(LEN(TRIM(B16))&gt;0,LEN(TRIM(C16))&gt;0,LEN(TRIM(D16))&gt;0,LEN(TRIM(E16))&gt;0),"Looks good","Add how you checked it"),IF(F16="Doesn't work",IF(LEN(TRIM(G16))&gt;0,"Needs fixing","Add next step"),IF(OR(F16="",F16="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I16" s="16">
         <f>IF(H16="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="17" ht="102" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Access and ownership</t>
+          <t>Other people's access</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Fictional replacement coordinator</t>
+          <t>Replacement coordinator</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Open the destination folder using their own account</t>
+          <t>Open the new folder using their own account</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
@@ -2610,12 +2561,12 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Receiver checked the exact destination, 16 Sep 2026</t>
+          <t>Other person checked the exact new folder, 16 Sep 2026</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Doesn't work</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -2623,19 +2574,19 @@
           <t>Grant the appropriate access and repeat the test. Do not share passwords.</t>
         </is>
       </c>
-      <c r="H17" s="15" t="str">
-        <f>IF(LEN(TRIM(A17&amp;B17&amp;C17&amp;D17&amp;E17&amp;F17&amp;G17))=0,"",IF(LEN(TRIM(A17))=0,"Name the check",IF(F17="Not applicable",IF(LEN(TRIM(G17))&gt;0,"Excluded by user","Explain exclusion"),IF(F17="Pass",IF(AND(LEN(TRIM(B17))&gt;0,LEN(TRIM(C17))&gt;0,LEN(TRIM(D17))&gt;0,LEN(TRIM(E17))&gt;0),"Pass recorded","Evidence missing"),IF(F17="Fail",IF(LEN(TRIM(G17))&gt;0,"Follow up","Add next action"),IF(OR(F17="",F17="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Follow up</v>
-      </c>
-      <c r="I17" s="16" t="n">
+      <c r="H17" s="15">
+        <f>IF(LEN(TRIM(A17&amp;B17&amp;C17&amp;D17&amp;E17&amp;F17&amp;G17))=0,"",IF(LEN(TRIM(A17))=0,"Name what you are checking",IF(F17="Doesn't apply",IF(LEN(TRIM(G17))&gt;0,"Doesn't apply","Say why"),IF(F17="Works",IF(AND(LEN(TRIM(B17))&gt;0,LEN(TRIM(C17))&gt;0,LEN(TRIM(D17))&gt;0,LEN(TRIM(E17))&gt;0),"Looks good","Add how you checked it"),IF(F17="Doesn't work",IF(LEN(TRIM(G17))&gt;0,"Needs fixing","Add next step"),IF(OR(F17="",F17="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I17" s="16">
         <f>IF(H17="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="18" ht="102" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>Scope and exceptions</t>
+          <t>Missing or skipped items</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2655,32 +2606,32 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Compared selected export scope with source inventory</t>
+          <t>Compared what was exported with the known list of items</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Doesn't work</t>
         </is>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>Resolve scope before relying on the export.</t>
-        </is>
-      </c>
-      <c r="H18" s="15" t="str">
-        <f>IF(LEN(TRIM(A18&amp;B18&amp;C18&amp;D18&amp;E18&amp;F18&amp;G18))=0,"",IF(LEN(TRIM(A18))=0,"Name the check",IF(F18="Not applicable",IF(LEN(TRIM(G18))&gt;0,"Excluded by user","Explain exclusion"),IF(F18="Pass",IF(AND(LEN(TRIM(B18))&gt;0,LEN(TRIM(C18))&gt;0,LEN(TRIM(D18))&gt;0,LEN(TRIM(E18))&gt;0),"Pass recorded","Evidence missing"),IF(F18="Fail",IF(LEN(TRIM(G18))&gt;0,"Follow up","Add next action"),IF(OR(F18="",F18="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Follow up</v>
-      </c>
-      <c r="I18" s="16" t="n">
+          <t>Export the missing item or confirm where it will live before relying on this copy.</t>
+        </is>
+      </c>
+      <c r="H18" s="15">
+        <f>IF(LEN(TRIM(A18&amp;B18&amp;C18&amp;D18&amp;E18&amp;F18&amp;G18))=0,"",IF(LEN(TRIM(A18))=0,"Name what you are checking",IF(F18="Doesn't apply",IF(LEN(TRIM(G18))&gt;0,"Doesn't apply","Say why"),IF(F18="Works",IF(AND(LEN(TRIM(B18))&gt;0,LEN(TRIM(C18))&gt;0,LEN(TRIM(D18))&gt;0,LEN(TRIM(E18))&gt;0),"Looks good","Add how you checked it"),IF(F18="Doesn't work",IF(LEN(TRIM(G18))&gt;0,"Needs fixing","Add next step"),IF(OR(F18="",F18="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I18" s="16">
         <f>IF(H18="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="19" ht="102" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>One real next action</t>
+          <t>One real thing I need to do</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2700,26 +2651,26 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Dry run stopped; no actual equipment move performed</t>
+          <t>The coordinator could not finish because the photo was missing</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Doesn't work</t>
         </is>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>Repeat only after the photo and its access are verified.</t>
-        </is>
-      </c>
-      <c r="H19" s="15" t="str">
-        <f>IF(LEN(TRIM(A19&amp;B19&amp;C19&amp;D19&amp;E19&amp;F19&amp;G19))=0,"",IF(LEN(TRIM(A19))=0,"Name the check",IF(F19="Not applicable",IF(LEN(TRIM(G19))&gt;0,"Excluded by user","Explain exclusion"),IF(F19="Pass",IF(AND(LEN(TRIM(B19))&gt;0,LEN(TRIM(C19))&gt;0,LEN(TRIM(D19))&gt;0,LEN(TRIM(E19))&gt;0),"Pass recorded","Evidence missing"),IF(F19="Fail",IF(LEN(TRIM(G19))&gt;0,"Follow up","Add next action"),IF(OR(F19="",F19="Not tested"),"Not tested","Check status"))))))</f>
-        <v>Follow up</v>
-      </c>
-      <c r="I19" s="16" t="n">
+          <t>Fix the photo and access, then try the task again.</t>
+        </is>
+      </c>
+      <c r="H19" s="15">
+        <f>IF(LEN(TRIM(A19&amp;B19&amp;C19&amp;D19&amp;E19&amp;F19&amp;G19))=0,"",IF(LEN(TRIM(A19))=0,"Name what you are checking",IF(F19="Doesn't apply",IF(LEN(TRIM(G19))&gt;0,"Doesn't apply","Say why"),IF(F19="Works",IF(AND(LEN(TRIM(B19))&gt;0,LEN(TRIM(C19))&gt;0,LEN(TRIM(D19))&gt;0,LEN(TRIM(E19))&gt;0),"Looks good","Add how you checked it"),IF(F19="Doesn't work",IF(LEN(TRIM(G19))&gt;0,"Needs fixing","Add next step"),IF(OR(F19="",F19="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I19" s="16">
         <f>IF(H19="",0,1)</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="20" ht="102" customHeight="1">
@@ -2730,13 +2681,13 @@
       <c r="E20" s="14" t="n"/>
       <c r="F20" s="14" t="n"/>
       <c r="G20" s="14" t="n"/>
-      <c r="H20" s="15" t="str">
-        <f>IF(LEN(TRIM(A20&amp;B20&amp;C20&amp;D20&amp;E20&amp;F20&amp;G20))=0,"",IF(LEN(TRIM(A20))=0,"Name the check",IF(F20="Not applicable",IF(LEN(TRIM(G20))&gt;0,"Excluded by user","Explain exclusion"),IF(F20="Pass",IF(AND(LEN(TRIM(B20))&gt;0,LEN(TRIM(C20))&gt;0,LEN(TRIM(D20))&gt;0,LEN(TRIM(E20))&gt;0),"Pass recorded","Evidence missing"),IF(F20="Fail",IF(LEN(TRIM(G20))&gt;0,"Follow up","Add next action"),IF(OR(F20="",F20="Not tested"),"Not tested","Check status"))))))</f>
-        <v/>
-      </c>
-      <c r="I20" s="16" t="n">
+      <c r="H20" s="15">
+        <f>IF(LEN(TRIM(A20&amp;B20&amp;C20&amp;D20&amp;E20&amp;F20&amp;G20))=0,"",IF(LEN(TRIM(A20))=0,"Name what you are checking",IF(F20="Doesn't apply",IF(LEN(TRIM(G20))&gt;0,"Doesn't apply","Say why"),IF(F20="Works",IF(AND(LEN(TRIM(B20))&gt;0,LEN(TRIM(C20))&gt;0,LEN(TRIM(D20))&gt;0,LEN(TRIM(E20))&gt;0),"Looks good","Add how you checked it"),IF(F20="Doesn't work",IF(LEN(TRIM(G20))&gt;0,"Needs fixing","Add next step"),IF(OR(F20="",F20="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I20" s="16">
         <f>IF(H20="",0,1)</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="21" ht="102" customHeight="1">
@@ -2747,13 +2698,13 @@
       <c r="E21" s="14" t="n"/>
       <c r="F21" s="14" t="n"/>
       <c r="G21" s="14" t="n"/>
-      <c r="H21" s="15" t="str">
-        <f>IF(LEN(TRIM(A21&amp;B21&amp;C21&amp;D21&amp;E21&amp;F21&amp;G21))=0,"",IF(LEN(TRIM(A21))=0,"Name the check",IF(F21="Not applicable",IF(LEN(TRIM(G21))&gt;0,"Excluded by user","Explain exclusion"),IF(F21="Pass",IF(AND(LEN(TRIM(B21))&gt;0,LEN(TRIM(C21))&gt;0,LEN(TRIM(D21))&gt;0,LEN(TRIM(E21))&gt;0),"Pass recorded","Evidence missing"),IF(F21="Fail",IF(LEN(TRIM(G21))&gt;0,"Follow up","Add next action"),IF(OR(F21="",F21="Not tested"),"Not tested","Check status"))))))</f>
-        <v/>
-      </c>
-      <c r="I21" s="16" t="n">
+      <c r="H21" s="15">
+        <f>IF(LEN(TRIM(A21&amp;B21&amp;C21&amp;D21&amp;E21&amp;F21&amp;G21))=0,"",IF(LEN(TRIM(A21))=0,"Name what you are checking",IF(F21="Doesn't apply",IF(LEN(TRIM(G21))&gt;0,"Doesn't apply","Say why"),IF(F21="Works",IF(AND(LEN(TRIM(B21))&gt;0,LEN(TRIM(C21))&gt;0,LEN(TRIM(D21))&gt;0,LEN(TRIM(E21))&gt;0),"Looks good","Add how you checked it"),IF(F21="Doesn't work",IF(LEN(TRIM(G21))&gt;0,"Needs fixing","Add next step"),IF(OR(F21="",F21="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I21" s="16">
         <f>IF(H21="",0,1)</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="22" ht="102" customHeight="1">
@@ -2764,13 +2715,13 @@
       <c r="E22" s="14" t="n"/>
       <c r="F22" s="14" t="n"/>
       <c r="G22" s="14" t="n"/>
-      <c r="H22" s="15" t="str">
-        <f>IF(LEN(TRIM(A22&amp;B22&amp;C22&amp;D22&amp;E22&amp;F22&amp;G22))=0,"",IF(LEN(TRIM(A22))=0,"Name the check",IF(F22="Not applicable",IF(LEN(TRIM(G22))&gt;0,"Excluded by user","Explain exclusion"),IF(F22="Pass",IF(AND(LEN(TRIM(B22))&gt;0,LEN(TRIM(C22))&gt;0,LEN(TRIM(D22))&gt;0,LEN(TRIM(E22))&gt;0),"Pass recorded","Evidence missing"),IF(F22="Fail",IF(LEN(TRIM(G22))&gt;0,"Follow up","Add next action"),IF(OR(F22="",F22="Not tested"),"Not tested","Check status"))))))</f>
-        <v/>
-      </c>
-      <c r="I22" s="16" t="n">
+      <c r="H22" s="15">
+        <f>IF(LEN(TRIM(A22&amp;B22&amp;C22&amp;D22&amp;E22&amp;F22&amp;G22))=0,"",IF(LEN(TRIM(A22))=0,"Name what you are checking",IF(F22="Doesn't apply",IF(LEN(TRIM(G22))&gt;0,"Doesn't apply","Say why"),IF(F22="Works",IF(AND(LEN(TRIM(B22))&gt;0,LEN(TRIM(C22))&gt;0,LEN(TRIM(D22))&gt;0,LEN(TRIM(E22))&gt;0),"Looks good","Add how you checked it"),IF(F22="Doesn't work",IF(LEN(TRIM(G22))&gt;0,"Needs fixing","Add next step"),IF(OR(F22="",F22="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I22" s="16">
         <f>IF(H22="",0,1)</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="23" ht="102" customHeight="1">
@@ -2781,13 +2732,13 @@
       <c r="E23" s="14" t="n"/>
       <c r="F23" s="14" t="n"/>
       <c r="G23" s="14" t="n"/>
-      <c r="H23" s="15" t="str">
-        <f>IF(LEN(TRIM(A23&amp;B23&amp;C23&amp;D23&amp;E23&amp;F23&amp;G23))=0,"",IF(LEN(TRIM(A23))=0,"Name the check",IF(F23="Not applicable",IF(LEN(TRIM(G23))&gt;0,"Excluded by user","Explain exclusion"),IF(F23="Pass",IF(AND(LEN(TRIM(B23))&gt;0,LEN(TRIM(C23))&gt;0,LEN(TRIM(D23))&gt;0,LEN(TRIM(E23))&gt;0),"Pass recorded","Evidence missing"),IF(F23="Fail",IF(LEN(TRIM(G23))&gt;0,"Follow up","Add next action"),IF(OR(F23="",F23="Not tested"),"Not tested","Check status"))))))</f>
-        <v/>
-      </c>
-      <c r="I23" s="16" t="n">
+      <c r="H23" s="15">
+        <f>IF(LEN(TRIM(A23&amp;B23&amp;C23&amp;D23&amp;E23&amp;F23&amp;G23))=0,"",IF(LEN(TRIM(A23))=0,"Name what you are checking",IF(F23="Doesn't apply",IF(LEN(TRIM(G23))&gt;0,"Doesn't apply","Say why"),IF(F23="Works",IF(AND(LEN(TRIM(B23))&gt;0,LEN(TRIM(C23))&gt;0,LEN(TRIM(D23))&gt;0,LEN(TRIM(E23))&gt;0),"Looks good","Add how you checked it"),IF(F23="Doesn't work",IF(LEN(TRIM(G23))&gt;0,"Needs fixing","Add next step"),IF(OR(F23="",F23="Not checked"),"Not checked","Check result"))))))</f>
+        <v/>
+      </c>
+      <c r="I23" s="16">
         <f>IF(H23="",0,1)</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -2803,16 +2754,9 @@
     <row r="25" ht="35" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>A recorded pass is your observation, not automatic verification. Test permissions using the intended receiver. Do not paste credentials or sensitive source records. Four blank rows allow additional checks.</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
+          <t>This example is invented. It shows why a downloaded export can look fine while an important file, link or permission still breaks the real task.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -3143,7 +3087,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="F11:F23" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Choose a listed result" error="Use Not tested, Pass, Fail or Not applicable." promptTitle="Record only what you checked" prompt="Pass needs a sample, expected and actual behaviour, plus evidence. An exclusion needs a reason." type="list" errorStyle="stop">
-      <formula1>"Not tested,Pass,Fail,Not applicable"</formula1>
+      <formula1>"Not checked,Works,Doesn't work,Doesn't apply"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>
@@ -3156,12 +3100,12 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <legacyDrawing ns1:id="anysvml"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0043161E"/>
     <outlinePr summaryBelow="1" summaryRight="0"/>
@@ -3186,13 +3130,6 @@
           <t>Eterna Clarity</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -3207,16 +3144,9 @@
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Sources, limits and reuse</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
+          <t>Sources and limits</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -3231,7 +3161,7 @@
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Version 1.0.0 | Published edition prepared 16 September 2026 | This is an organisational worksheet, not a backup, restore engine, compliance audit or security assessment.</t>
+          <t>Version 1.1.0 | Updated 16 September 2026 | This checklist helps you test an export. It is not backup software, a security audit, or legal/compliance advice.</t>
         </is>
       </c>
     </row>
@@ -3251,13 +3181,6 @@
           <t>Notion backup documentation</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8" ht="27" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
@@ -3269,7 +3192,7 @@
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>An export is not an instant reconstruction of the original workspace. This is one product-specific example of why the destination must be tested.</t>
+          <t>An export may give you readable files without recreating the original workspace. This is one example of why it is worth testing what you actually need to do.</t>
         </is>
       </c>
     </row>
@@ -3289,13 +3212,6 @@
           <t>Notion Mail transition notice</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12" ht="27" customHeight="1">
       <c r="A12" s="17" t="inlineStr">
@@ -3307,7 +3223,7 @@
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>The 2026 transition distinguishes synced email history from app-only data and settings. Use current provider instructions for actual deadlines and export steps.</t>
+          <t>The 2026 transition separates synced email history from some app-only information and settings. Use the app’s current instructions for any real deadlines or export steps.</t>
         </is>
       </c>
     </row>
@@ -3327,13 +3243,6 @@
           <t>Google Drive ownership transfer</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16" ht="27" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
@@ -3345,7 +3254,7 @@
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Changing a folder owner does not change ownership of files within it. Check the actual objects and receiver access.</t>
+          <t>Changing who owns a folder does not automatically change ownership of every file inside it. Check the files and the other person's actual access.</t>
         </is>
       </c>
     </row>
@@ -3372,28 +3281,21 @@
     <row r="20" ht="29" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Boundaries</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
+          <t>Important limits</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="43" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>The worksheet does not inspect your source or destination. It cannot prove completeness, restore unsupported features, check legal retention requirements or decide when it is safe to delete an account. A small sample is not exhaustive validation.</t>
+          <t>This workbook does not inspect your files automatically. It cannot prove that every item was exported, restore missing app features, check legal retention requirements, or decide when it is safe to delete an account.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="43" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Follow current provider instructions and your organisation's rules. Use isolated test data where possible. A source or destination may restrict export, imports, ownership transfers or sharing. Resolve such limits with the relevant owner.</t>
+          <t>Follow the current instructions for the app you are leaving and the place you are moving to. Test with copies where possible, keep the originals, and check sharing or access before you rely on the new copy.</t>
         </is>
       </c>
     </row>
@@ -3413,25 +3315,18 @@
           <t>Licence</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
     </row>
     <row r="25" ht="43" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Original worksheet prose, blank template, fictional example and workbook content: Creative Commons Attribution 4.0 International (CC BY 4.0). Eterna names/logos/trademarks and linked third-party material are not included in this grant.</t>
+          <t>Original checklist text, blank template, fictional example and workbook content: Creative Commons Attribution 4.0 International (CC BY 4.0). Eterna names, logos, trademarks and linked third-party material are not included in this licence.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Attribution: Export and Recovery Rehearsal by Eterna Clarity, licensed under CC BY 4.0. Licence: https://creativecommons.org/licenses/by/4.0/</t>
+          <t>Attribution: Export Check: Can I Still Use My Data? by Eterna Clarity, licensed under CC BY 4.0. Licence: https://creativecommons.org/licenses/by/4.0/</t>
         </is>
       </c>
     </row>
@@ -3727,12 +3622,12 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A25:H25"/>
@@ -3747,10 +3642,10 @@
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A8" ns1:id="rId1"/>
-    <hyperlink ref="A12" ns1:id="rId2"/>
-    <hyperlink ref="A16" ns1:id="rId3"/>
-    <hyperlink ref="A26" ns1:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>